<commit_message>
Fill warehouse address ids from warehouse codes
</commit_message>
<xml_diff>
--- a/docs/manual-fill/Warehouses_Missing_Fields_To_Fill_simple.xlsx
+++ b/docs/manual-fill/Warehouses_Missing_Fields_To_Fill_simple.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -67,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -76,6 +81,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -531,15 +539,31 @@
           <t>CC8 - ACER - MAIN - JHB - SPL</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr"/>
-      <c r="K2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ACER</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="inlineStr"/>
+      <c r="I2" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4" t="inlineStr"/>
+      <c r="K2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -552,15 +576,31 @@
           <t>CC8 - ACER - KHAULEZA - JHB - SPL - OFFSITE</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ACERKH</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -573,15 +613,31 @@
           <t>CC8 - BNI - CPT - ONSITE</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>BNI CT</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -594,15 +650,27 @@
           <t>CHOICE LOGISTICS CT W/H</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>CHLCT</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -615,15 +683,27 @@
           <t>CHOICE LOGISTICS MAIN W/H</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>CHLJHB</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr"/>
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -636,15 +716,27 @@
           <t>Choice Logistics Warehouse</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>CHOICE</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -657,15 +749,23 @@
           <t>FRANCOIS TRANSIT TO CT</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>FRANCOIS</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -678,15 +778,27 @@
           <t>CC8 - MAIN - GREEN - JHB - SPL</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>FSCGREEN</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -699,15 +811,27 @@
           <t>FUJ GREEN STOCK CT</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="3" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>FSCGRNCT</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -720,15 +844,27 @@
           <t>CC8 - TRACKER - JHB - ONSITE</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>FSCTRAC</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -741,15 +877,27 @@
           <t>CC8 - MAIN - CPT - SPL</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>FUJ CT</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -762,15 +910,27 @@
           <t>CC8 - MAIN - KZN - SPL</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>FUJ DBN</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -783,15 +943,27 @@
           <t>CC8 - FUJ - IEC</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr"/>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr"/>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>FUJ IEC</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -804,15 +976,27 @@
           <t>CC8 - LUFTHANZA - JHB - SPL</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>FUJ LUFT</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -825,15 +1009,27 @@
           <t>CC8 - IPTH - NC - ONSITE</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr"/>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="3" t="inlineStr"/>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
-      <c r="J16" s="3" t="inlineStr"/>
-      <c r="K16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>FUJ PETR</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -846,15 +1042,27 @@
           <t>CC8 - ROYAL SWAZI SUGAR - SWAZI - ONSITE</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr"/>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr"/>
-      <c r="J17" s="3" t="inlineStr"/>
-      <c r="K17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>FUJ RSSC</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -867,15 +1075,27 @@
           <t>CC8 - TOYOTA - KZN - ONSITE</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr"/>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr"/>
-      <c r="K18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>FUJ TYT</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -888,15 +1108,23 @@
           <t>CC8 - DOA - JHB - SPL</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr"/>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="3" t="inlineStr"/>
-      <c r="K19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>FUJDOA</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr"/>
+      <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -909,15 +1137,23 @@
           <t>CC8 - FAULTY RETURN TO GERMANY FOR CREDIT - JHB - SPL</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr"/>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr"/>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="3" t="inlineStr"/>
-      <c r="K20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -930,15 +1166,27 @@
           <t>CC8 - H&amp;M - CPT - SPL</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr"/>
-      <c r="J21" s="3" t="inlineStr"/>
-      <c r="K21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>FUJH&amp;M-C</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -951,15 +1199,27 @@
           <t>CC8 - H&amp;M - JHB - SPL</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr"/>
-      <c r="D22" s="3" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr"/>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr"/>
-      <c r="J22" s="3" t="inlineStr"/>
-      <c r="K22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>FUJH&amp;M-J</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr"/>
+      <c r="H22" s="4" t="inlineStr"/>
+      <c r="I22" s="4" t="inlineStr"/>
+      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -972,15 +1232,27 @@
           <t>CC8 - MAIN - JHB - SPL</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr"/>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr"/>
-      <c r="K23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -993,15 +1265,27 @@
           <t>CC8 - MIWAY - JHB - TBI</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr"/>
-      <c r="D24" s="3" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr"/>
-      <c r="G24" s="3" t="inlineStr"/>
-      <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr"/>
-      <c r="J24" s="3" t="inlineStr"/>
-      <c r="K24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>FUJMIW-J</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1014,15 +1298,27 @@
           <t>CC8 - MASSMART - CPT - SPL</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr"/>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr"/>
-      <c r="J25" s="3" t="inlineStr"/>
-      <c r="K25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>FUJMSM C</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1035,15 +1331,27 @@
           <t>CC8 - MASSMART - JHB - SPL- LOCATED AT COCRE8</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr"/>
-      <c r="D26" s="3" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr"/>
-      <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr"/>
-      <c r="I26" s="3" t="inlineStr"/>
-      <c r="J26" s="3" t="inlineStr"/>
-      <c r="K26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>FUJMSM J</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr"/>
+      <c r="H26" s="4" t="inlineStr"/>
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1056,15 +1364,27 @@
           <t>CC8 - MASSMART - VCF - JHB - SPL</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr"/>
-      <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr"/>
-      <c r="J27" s="3" t="inlineStr"/>
-      <c r="K27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>FUJMSVCJ</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr"/>
+      <c r="H27" s="4" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1077,15 +1397,23 @@
           <t>CC8 - NON RETURNABLE / SCRAP PART - JHB - SPL</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr"/>
-      <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr"/>
-      <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>FUJNRP</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr"/>
+      <c r="H28" s="4" t="inlineStr"/>
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1098,15 +1426,27 @@
           <t>CC8 - OLD MUTUAL - CPT - TBI</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="3" t="inlineStr"/>
-      <c r="I29" s="3" t="inlineStr"/>
-      <c r="J29" s="3" t="inlineStr"/>
-      <c r="K29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>FUJOM CT</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr"/>
+      <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1119,15 +1459,27 @@
           <t>CC8 - MAIN - EC - TBI</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr"/>
-      <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="3" t="inlineStr"/>
-      <c r="G30" s="3" t="inlineStr"/>
-      <c r="H30" s="3" t="inlineStr"/>
-      <c r="I30" s="3" t="inlineStr"/>
-      <c r="J30" s="3" t="inlineStr"/>
-      <c r="K30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>FUJPE</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr"/>
+      <c r="H30" s="4" t="inlineStr"/>
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1140,15 +1492,27 @@
           <t>CC8 - SANLAM - CPT - TBI</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr"/>
-      <c r="G31" s="3" t="inlineStr"/>
-      <c r="H31" s="3" t="inlineStr"/>
-      <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="inlineStr"/>
-      <c r="K31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>FUJSANCT</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1161,15 +1525,27 @@
           <t>CC8 - DATASIENCES FOR STANDARD BANK - TBI - TBI</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr"/>
-      <c r="D32" s="3" t="inlineStr"/>
-      <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr"/>
-      <c r="G32" s="3" t="inlineStr"/>
-      <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr"/>
-      <c r="J32" s="3" t="inlineStr"/>
-      <c r="K32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>FUJSTDBN</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="4" t="inlineStr"/>
+      <c r="I32" s="4" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1182,15 +1558,27 @@
           <t>CC8 - SWAZI BANK - SWAZI - ONSITE</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr"/>
-      <c r="J33" s="3" t="inlineStr"/>
-      <c r="K33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>FUJSWBAN</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr"/>
+      <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1203,15 +1591,27 @@
           <t>CC8 - SIZWE WESTERN CAPE - WC - TBI</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr"/>
-      <c r="D34" s="3" t="inlineStr"/>
-      <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="3" t="inlineStr"/>
-      <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr"/>
-      <c r="J34" s="3" t="inlineStr"/>
-      <c r="K34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>FUJSWWC</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr"/>
+      <c r="H34" s="4" t="inlineStr"/>
+      <c r="I34" s="4" t="inlineStr"/>
+      <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1224,15 +1624,23 @@
           <t>CC8 - UNUSED PART RETURNS TO GO BACK TO FUJ MAIN - JHB - SPL</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr"/>
-      <c r="G35" s="3" t="inlineStr"/>
-      <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr"/>
-      <c r="J35" s="3" t="inlineStr"/>
-      <c r="K35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>FUJUNUSE</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr"/>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1245,15 +1653,23 @@
           <t>CC8 - STK WRITE OFF - TBI - TBI</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr"/>
-      <c r="D36" s="3" t="inlineStr"/>
-      <c r="E36" s="3" t="inlineStr"/>
-      <c r="F36" s="3" t="inlineStr"/>
-      <c r="G36" s="3" t="inlineStr"/>
-      <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr"/>
-      <c r="J36" s="3" t="inlineStr"/>
-      <c r="K36" s="3" t="inlineStr"/>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>FUJWO</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr"/>
+      <c r="H36" s="4" t="inlineStr"/>
+      <c r="I36" s="4" t="inlineStr"/>
+      <c r="J36" s="4" t="inlineStr"/>
+      <c r="K36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1266,15 +1682,23 @@
           <t>CC8 - WRITE OFF - CPT - SPL</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr"/>
-      <c r="G37" s="3" t="inlineStr"/>
-      <c r="H37" s="3" t="inlineStr"/>
-      <c r="I37" s="3" t="inlineStr"/>
-      <c r="J37" s="3" t="inlineStr"/>
-      <c r="K37" s="3" t="inlineStr"/>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>FUJWO CT</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1287,15 +1711,23 @@
           <t>CC8 - RESC WRITE OFF - TBI - TBI</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr"/>
-      <c r="D38" s="3" t="inlineStr"/>
-      <c r="E38" s="3" t="inlineStr"/>
-      <c r="F38" s="3" t="inlineStr"/>
-      <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="3" t="inlineStr"/>
-      <c r="J38" s="3" t="inlineStr"/>
-      <c r="K38" s="3" t="inlineStr"/>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>FUJWORSS</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr"/>
+      <c r="H38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr"/>
+      <c r="J38" s="4" t="inlineStr"/>
+      <c r="K38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1308,15 +1740,27 @@
           <t>Choice RMA Warehouse</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr"/>
-      <c r="G39" s="3" t="inlineStr"/>
-      <c r="H39" s="3" t="inlineStr"/>
-      <c r="I39" s="3" t="inlineStr"/>
-      <c r="J39" s="3" t="inlineStr"/>
-      <c r="K39" s="3" t="inlineStr"/>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>GCJRMA</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr"/>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1329,15 +1773,23 @@
           <t>FORTINET FAULTY WAREHOUSE</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr"/>
-      <c r="D40" s="3" t="inlineStr"/>
-      <c r="E40" s="3" t="inlineStr"/>
-      <c r="F40" s="3" t="inlineStr"/>
-      <c r="G40" s="3" t="inlineStr"/>
-      <c r="H40" s="3" t="inlineStr"/>
-      <c r="I40" s="3" t="inlineStr"/>
-      <c r="J40" s="3" t="inlineStr"/>
-      <c r="K40" s="3" t="inlineStr"/>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>MF FAULT</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr"/>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr"/>
+      <c r="J40" s="4" t="inlineStr"/>
+      <c r="K40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1350,15 +1802,27 @@
           <t>Maxtec Waehouse</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr"/>
-      <c r="G41" s="3" t="inlineStr"/>
-      <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr"/>
-      <c r="J41" s="3" t="inlineStr"/>
-      <c r="K41" s="3" t="inlineStr"/>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>MXT</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr"/>
+      <c r="K41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1371,15 +1835,23 @@
           <t>CC8 - QUARANTINE - JHB - SPL</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr"/>
-      <c r="D42" s="3" t="inlineStr"/>
-      <c r="E42" s="3" t="inlineStr"/>
-      <c r="F42" s="3" t="inlineStr"/>
-      <c r="G42" s="3" t="inlineStr"/>
-      <c r="H42" s="3" t="inlineStr"/>
-      <c r="I42" s="3" t="inlineStr"/>
-      <c r="J42" s="3" t="inlineStr"/>
-      <c r="K42" s="3" t="inlineStr"/>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>QURN</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr"/>
+      <c r="J42" s="4" t="inlineStr"/>
+      <c r="K42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1392,15 +1864,23 @@
           <t>FUJITSU SCRAP QUEUE</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr"/>
-      <c r="G43" s="3" t="inlineStr"/>
-      <c r="H43" s="3" t="inlineStr"/>
-      <c r="I43" s="3" t="inlineStr"/>
-      <c r="J43" s="3" t="inlineStr"/>
-      <c r="K43" s="3" t="inlineStr"/>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>SCRPFUJ</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr"/>
+      <c r="K43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1413,15 +1893,23 @@
           <t>CC8 - SIZWE QUARANTINE - TBI - TBI</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr"/>
-      <c r="D44" s="3" t="inlineStr"/>
-      <c r="E44" s="3" t="inlineStr"/>
-      <c r="F44" s="3" t="inlineStr"/>
-      <c r="G44" s="3" t="inlineStr"/>
-      <c r="H44" s="3" t="inlineStr"/>
-      <c r="I44" s="3" t="inlineStr"/>
-      <c r="J44" s="3" t="inlineStr"/>
-      <c r="K44" s="3" t="inlineStr"/>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>SIZ-QURN</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="4" t="inlineStr"/>
+      <c r="K44" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -1453,108 +1941,108 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>What to Fill</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>addressId</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Address/site id linking this warehouse to Addresses.csv. Leave blank if we are not using Addresses for MVP.</t>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Derived from warehouseId / SAP warehouse code per user mapping. Example: FUJ CT.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>returnWarehouseId</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Preferred warehouse for returned/faulty parts. Use a warehouseId from the WarehouseIds sheet, or N/A.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>supplyWarehouseId</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Preferred replenishment/source warehouse. Use a warehouseId from the WarehouseIds sheet, or N/A.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>warehouseTypeId</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Planning warehouse type. Examples in template are BOOT, DEP, REPAIR. Use a short controlled value we can standardise later.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>isReplenishable</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>TRUE if this warehouse should be replenished by the planning engine; FALSE/N/A otherwise.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>isBranchStockable</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>TRUE if this branch/location can hold branch stock; FALSE/N/A otherwise.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>isRemote</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>TRUE if this is an outlying/remote location; FALSE/N/A otherwise.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>warehouseStatusId</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Active/inactive/obsolete status. Suggested values: ACTIVE, INACTIVE, OBSOLETE, N/A.</t>
         </is>
@@ -1579,12 +2067,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>warehouseId</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>warehouseDescription</t>
         </is>

</xml_diff>

<commit_message>
Restore warehouse fill rows for obsolete review
</commit_message>
<xml_diff>
--- a/docs/manual-fill/Warehouses_Missing_Fields_To_Fill_simple.xlsx
+++ b/docs/manual-fill/Warehouses_Missing_Fields_To_Fill_simple.xlsx
@@ -72,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -86,7 +86,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -455,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -468,7 +467,9 @@
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,6 +525,16 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>isObsolete</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>activityEvidence</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -555,15 +566,21 @@
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr"/>
-      <c r="G2" s="4" t="b">
-        <v>1</v>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="4" t="b">
-        <v>0</v>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
       <c r="J2" s="4" t="inlineStr"/>
       <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr"/>
+      <c r="M2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -592,15 +609,21 @@
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr"/>
-      <c r="G3" s="4" t="b">
-        <v>1</v>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="4" t="b">
-        <v>1</v>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
       <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr"/>
+      <c r="M3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -629,15 +652,21 @@
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr"/>
-      <c r="G4" s="4" t="b">
-        <v>1</v>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="b">
-        <v>1</v>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -671,6 +700,8 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -704,6 +735,8 @@
       <c r="I6" s="4" t="inlineStr"/>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -737,6 +770,8 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr"/>
+      <c r="M7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -766,6 +801,8 @@
       <c r="I8" s="4" t="inlineStr"/>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -799,6 +836,8 @@
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -832,6 +871,8 @@
       <c r="I10" s="4" t="inlineStr"/>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -865,6 +906,8 @@
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
+      <c r="M11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -898,6 +941,8 @@
       <c r="I12" s="4" t="inlineStr"/>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -931,6 +976,8 @@
       <c r="I13" s="4" t="inlineStr"/>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -964,6 +1011,8 @@
       <c r="I14" s="4" t="inlineStr"/>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -997,6 +1046,8 @@
       <c r="I15" s="4" t="inlineStr"/>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1030,6 +1081,8 @@
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1063,6 +1116,8 @@
       <c r="I17" s="4" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1096,6 +1151,8 @@
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1125,6 +1182,8 @@
       <c r="I19" s="4" t="inlineStr"/>
       <c r="J19" s="4" t="inlineStr"/>
       <c r="K19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1154,6 +1213,8 @@
       <c r="I20" s="4" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1187,6 +1248,8 @@
       <c r="I21" s="4" t="inlineStr"/>
       <c r="J21" s="4" t="inlineStr"/>
       <c r="K21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr"/>
+      <c r="M21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1220,6 +1283,8 @@
       <c r="I22" s="4" t="inlineStr"/>
       <c r="J22" s="4" t="inlineStr"/>
       <c r="K22" s="4" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr"/>
+      <c r="M22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1253,6 +1318,8 @@
       <c r="I23" s="4" t="inlineStr"/>
       <c r="J23" s="4" t="inlineStr"/>
       <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1286,6 +1353,8 @@
       <c r="I24" s="4" t="inlineStr"/>
       <c r="J24" s="4" t="inlineStr"/>
       <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1319,6 +1388,8 @@
       <c r="I25" s="4" t="inlineStr"/>
       <c r="J25" s="4" t="inlineStr"/>
       <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr"/>
+      <c r="M25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1352,6 +1423,8 @@
       <c r="I26" s="4" t="inlineStr"/>
       <c r="J26" s="4" t="inlineStr"/>
       <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1385,6 +1458,8 @@
       <c r="I27" s="4" t="inlineStr"/>
       <c r="J27" s="4" t="inlineStr"/>
       <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
+      <c r="M27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1414,6 +1489,8 @@
       <c r="I28" s="4" t="inlineStr"/>
       <c r="J28" s="4" t="inlineStr"/>
       <c r="K28" s="4" t="inlineStr"/>
+      <c r="L28" s="4" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1447,6 +1524,8 @@
       <c r="I29" s="4" t="inlineStr"/>
       <c r="J29" s="4" t="inlineStr"/>
       <c r="K29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr"/>
+      <c r="M29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1480,6 +1559,8 @@
       <c r="I30" s="4" t="inlineStr"/>
       <c r="J30" s="4" t="inlineStr"/>
       <c r="K30" s="4" t="inlineStr"/>
+      <c r="L30" s="4" t="inlineStr"/>
+      <c r="M30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1513,6 +1594,8 @@
       <c r="I31" s="4" t="inlineStr"/>
       <c r="J31" s="4" t="inlineStr"/>
       <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr"/>
+      <c r="M31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1546,6 +1629,8 @@
       <c r="I32" s="4" t="inlineStr"/>
       <c r="J32" s="4" t="inlineStr"/>
       <c r="K32" s="4" t="inlineStr"/>
+      <c r="L32" s="4" t="inlineStr"/>
+      <c r="M32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1579,6 +1664,8 @@
       <c r="I33" s="4" t="inlineStr"/>
       <c r="J33" s="4" t="inlineStr"/>
       <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr"/>
+      <c r="M33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1612,6 +1699,8 @@
       <c r="I34" s="4" t="inlineStr"/>
       <c r="J34" s="4" t="inlineStr"/>
       <c r="K34" s="4" t="inlineStr"/>
+      <c r="L34" s="4" t="inlineStr"/>
+      <c r="M34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1641,6 +1730,8 @@
       <c r="I35" s="4" t="inlineStr"/>
       <c r="J35" s="4" t="inlineStr"/>
       <c r="K35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr"/>
+      <c r="M35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1670,6 +1761,8 @@
       <c r="I36" s="4" t="inlineStr"/>
       <c r="J36" s="4" t="inlineStr"/>
       <c r="K36" s="4" t="inlineStr"/>
+      <c r="L36" s="4" t="inlineStr"/>
+      <c r="M36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1699,6 +1792,8 @@
       <c r="I37" s="4" t="inlineStr"/>
       <c r="J37" s="4" t="inlineStr"/>
       <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1728,6 +1823,8 @@
       <c r="I38" s="4" t="inlineStr"/>
       <c r="J38" s="4" t="inlineStr"/>
       <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="4" t="inlineStr"/>
+      <c r="M38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1761,6 +1858,8 @@
       <c r="I39" s="4" t="inlineStr"/>
       <c r="J39" s="4" t="inlineStr"/>
       <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr"/>
+      <c r="M39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1790,6 +1889,8 @@
       <c r="I40" s="4" t="inlineStr"/>
       <c r="J40" s="4" t="inlineStr"/>
       <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="4" t="inlineStr"/>
+      <c r="M40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1823,6 +1924,8 @@
       <c r="I41" s="4" t="inlineStr"/>
       <c r="J41" s="4" t="inlineStr"/>
       <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="4" t="inlineStr"/>
+      <c r="M41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1852,6 +1955,8 @@
       <c r="I42" s="4" t="inlineStr"/>
       <c r="J42" s="4" t="inlineStr"/>
       <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="4" t="inlineStr"/>
+      <c r="M42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1881,6 +1986,8 @@
       <c r="I43" s="4" t="inlineStr"/>
       <c r="J43" s="4" t="inlineStr"/>
       <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr"/>
+      <c r="M43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1910,9 +2017,11 @@
       <c r="I44" s="4" t="inlineStr"/>
       <c r="J44" s="4" t="inlineStr"/>
       <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="4" t="inlineStr"/>
+      <c r="M44" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="G2:G44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE,N/A"</formula1>
     </dataValidation>
@@ -1921,6 +2030,9 @@
     </dataValidation>
     <dataValidation sqref="I2:I44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Y,N,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1933,7 +2045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1941,110 +2053,134 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>What to Fill</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>addressId</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Derived from warehouseId / SAP warehouse code per user mapping. Example: FUJ CT.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>returnWarehouseId</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Preferred warehouse for returned/faulty parts. Use a warehouseId from the WarehouseIds sheet, or N/A.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>supplyWarehouseId</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Preferred replenishment/source warehouse. Use a warehouseId from the WarehouseIds sheet, or N/A.</t>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Preferred replenishment/source warehouse. Blank means virtual/quarantine/faulty-return warehouse and is excluded from MVP planning outputs.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>warehouseTypeId</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Planning warehouse type. Examples in template are BOOT, DEP, REPAIR. Use a short controlled value we can standardise later.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>isReplenishable</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>TRUE if this warehouse should be replenished by the planning engine; FALSE/N/A otherwise.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>isBranchStockable</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>TRUE if this branch/location can hold branch stock; FALSE/N/A otherwise.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>isRemote</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>TRUE if this is an outlying/remote location; FALSE/N/A otherwise.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>warehouseStatusId</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Active/inactive/obsolete status. Suggested values: ACTIVE, INACTIVE, OBSOLETE, N/A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>isObsolete</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Use Y when the warehouse/site is not being used, empty, or should not participate in planning. Use N for active planning warehouses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>activityEvidence</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Optional evidence/comment for recent stock movement or empty status. This is for review and is not a template field.</t>
         </is>
       </c>
     </row>
@@ -2062,533 +2198,533 @@
   <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>warehouseId</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>warehouseDescription</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>ACER</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>CC8 - ACER - MAIN - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>ACERKH</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>CC8 - ACER - KHAULEZA - JHB - SPL - OFFSITE</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>BNI CT</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>CC8 - BNI - CPT - ONSITE</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>CHLCT</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>CHOICE LOGISTICS CT W/H</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>CHLJHB</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>CHOICE LOGISTICS MAIN W/H</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>CHOICE</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Choice Logistics Warehouse</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>FRANCOIS</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>FRANCOIS TRANSIT TO CT</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>FSCGREEN</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>CC8 - MAIN - GREEN - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>FSCGRNCT</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>FUJ GREEN STOCK CT</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>FSCTRAC</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>CC8 - TRACKER - JHB - ONSITE</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>FUJ CT</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>CC8 - MAIN - CPT - SPL</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>FUJ DBN</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>CC8 - MAIN - KZN - SPL</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>FUJ IEC</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>CC8 - FUJ - IEC</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>FUJ LUFT</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>CC8 - LUFTHANZA - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>FUJ PETR</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>CC8 - IPTH - NC - ONSITE</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>FUJ RSSC</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>CC8 - ROYAL SWAZI SUGAR - SWAZI - ONSITE</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>FUJ TYT</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>CC8 - TOYOTA - KZN - ONSITE</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>FUJDOA</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>CC8 - DOA - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>FUJFAULT</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>FUJFAULT</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>CC8 - FAULTY RETURN TO GERMANY FOR CREDIT - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>FUJH&amp;M-C</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>CC8 - H&amp;M - CPT - SPL</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>FUJH&amp;M-J</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>CC8 - H&amp;M - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>FUJITSU</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>FUJITSU</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>CC8 - MAIN - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>FUJMIW-J</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>CC8 - MIWAY - JHB - TBI</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>FUJMSM C</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>CC8 - MASSMART - CPT - SPL</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>FUJMSM J</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>CC8 - MASSMART - JHB - SPL- LOCATED AT COCRE8</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>FUJMSVCJ</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>CC8 - MASSMART - VCF - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>FUJNRP</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>CC8 - NON RETURNABLE / SCRAP PART - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>FUJOM CT</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>CC8 - OLD MUTUAL - CPT - TBI</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>FUJPE</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>CC8 - MAIN - EC - TBI</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>FUJSANCT</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>CC8 - SANLAM - CPT - TBI</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>FUJSTDBN</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>CC8 - DATASIENCES FOR STANDARD BANK - TBI - TBI</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>FUJSWBAN</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>CC8 - SWAZI BANK - SWAZI - ONSITE</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>FUJSWWC</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>CC8 - SIZWE WESTERN CAPE - WC - TBI</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>FUJUNUSE</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>CC8 - UNUSED PART RETURNS TO GO BACK TO FUJ MAIN - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>FUJWO</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>CC8 - STK WRITE OFF - TBI - TBI</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>FUJWO CT</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>CC8 - WRITE OFF - CPT - SPL</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>FUJWORSS</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>CC8 - RESC WRITE OFF - TBI - TBI</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>GCJRMA</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Choice RMA Warehouse</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>MF FAULT</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>FORTINET FAULTY WAREHOUSE</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>MXT</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Maxtec Waehouse</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>QURN</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>CC8 - QUARANTINE - JHB - SPL</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>SCRPFUJ</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>FUJITSU SCRAP QUEUE</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>SIZ-QURN</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>CC8 - SIZWE QUARANTINE - TBI - TBI</t>
         </is>

</xml_diff>

<commit_message>
Complete warehouse obsolete flags
</commit_message>
<xml_diff>
--- a/docs/manual-fill/Warehouses_Missing_Fields_To_Fill_simple.xlsx
+++ b/docs/manual-fill/Warehouses_Missing_Fields_To_Fill_simple.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PlanningV2_CC8\docs\manual-fill\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCA3E428-9070-48EC-AF62-0574ED8F82E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA93A059-9619-4CED-942C-9366F3CD6B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30360" yWindow="1620" windowWidth="26760" windowHeight="13770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29745" yWindow="1320" windowWidth="26760" windowHeight="13770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Warehouses To Fill" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="117">
   <si>
     <t>warehouseId</t>
   </si>
@@ -1253,7 +1253,9 @@
       </c>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
+      <c r="K14" s="4" t="s">
+        <v>116</v>
+      </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4"/>
     </row>
@@ -1354,7 +1356,9 @@
         <v>1</v>
       </c>
       <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
+      <c r="K17" s="4" t="s">
+        <v>116</v>
+      </c>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
     </row>
@@ -1387,7 +1391,9 @@
         <v>0</v>
       </c>
       <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
+      <c r="K18" s="4" t="s">
+        <v>111</v>
+      </c>
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
     </row>
@@ -1589,7 +1595,9 @@
       </c>
       <c r="I24" s="4"/>
       <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
+      <c r="K24" s="4" t="s">
+        <v>111</v>
+      </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
     </row>
@@ -1865,7 +1873,9 @@
         <v>0</v>
       </c>
       <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
+      <c r="K32" s="4" t="s">
+        <v>116</v>
+      </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
     </row>
@@ -1898,7 +1908,9 @@
         <v>1</v>
       </c>
       <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
+      <c r="K33" s="4" t="s">
+        <v>116</v>
+      </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
     </row>
@@ -1931,7 +1943,9 @@
         <v>0</v>
       </c>
       <c r="J34" s="4"/>
-      <c r="K34" s="4"/>
+      <c r="K34" s="4" t="s">
+        <v>111</v>
+      </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
     </row>
@@ -2260,7 +2274,7 @@
       </c>
       <c r="J44" s="4"/>
       <c r="K44" s="4" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="L44" s="4"/>
       <c r="M44" s="4"/>

</xml_diff>